<commit_message>
Redesign PV mount to 3x4, sync tender package, fix rural-star-sjednica sim pipeline
PV mount redesign (2 supports x 6 modules -> 3 supports x 4 modules, raised
+0,50m -> +1,50m bottom edge) propagated through drawings (S-02/S-03/E-01),
BOQ, and Prilog I; two real bugs found and fixed in tools/rebuild_pdfs.py
(stale duplicate M-01/E-01 pages, obsolete Huawei catalogue reference pages).
tools/check_consistency.py now passes 0 failures across the whole package.

rural-star-sjednica: fixed three real bugs blocking the Radiance pipeline
from ever running (invalid 'box' primitive -> genbox/xform, sensor position
below the raised panel field, silently-discarded return type), added
incremental/resumable CSV output, switched PVLib transposition to Perez,
and added a PVGIS-TMY source option. Config synced to the actual 585W
module and 22kVA genset (was 540W/13.5kW).
</commit_message>
<xml_diff>
--- a/bht-sjednica-final-review/TD-OUTPUT/3.1 PRILOG II TD - predmjer Sjednica Bileca.xlsx
+++ b/bht-sjednica-final-review/TD-OUTPUT/3.1 PRILOG II TD - predmjer Sjednica Bileca.xlsx
@@ -1312,14 +1312,14 @@
       <c r="B12" s="80" t="inlineStr">
         <is>
           <t>Isporuka i montaža nosive metalne konstrukcije (ground mount support) za prihvat fotonaponskih panela, karakteristika:
- - tip: A-izvedba, NISKA izvedba (Standard A-Shaped Support 3.0 — LOW SUPPORT), kao Huawei BOM 21540481 sa ankerima BOM 21540482, antitheft maticom 21540036 i ključem 21540038, ili ekvivalent istih ili boljih karakteristika
+ - tip: CUSTOM IZRADA (izvan kataloga zbog opterećenja vjetrom, v. niže) — 3 nosača, svaki za 4 fotonaponska modula (2 reda × 2 kolone, portret); geometrija margina/prepusta preuzeta iz Huawei Standard A-Shaped Support 3.0 konvencije (PVM Tabela 4-20), ali poprečna greda izrađena po mjeri za 2 kolone modula, ne za kataloških 6
  - inklinacija: fiksno 45°, orijentacija JUG (azimut 180°). Nagib je zadržan zbog decembarskog prinosa — pri podnevnoj visini Sunca 23,6° na 42,94° N nagib 45° ostvaruje 93 % direktnog zračenja u odnosu na 85 % pri 35°, a decembar je mjerodavni mjesec za dimenzionisanje autonomnog sistema
- - gabariti PV polja (2 reda × 3 modula, portret): širina polja 3476 mm (poprečna greda 4089 mm, bočni prepust 306,5 mm), dužina polja po nagibu 4576 mm (2 × 2278 mm), horizontalna projekcija 3236 mm pri nagibu 45°; donja ivica panela na +0,50 m, gornja ivica na +3,74 m od nivoa terena
- - smještaj: nosač se temelji IZVAN ograđenog platoa, 1400 mm južno od kote ograde (raspoloživi pojas 1950 mm); gornja (sjeverna) ivica panela je 1,84 m iznad kote ograde h=1,90 m i prelazi preko platoa na visini +3,50 m, iznad krova kontejnera. Ponuđač provjerava da konstrukcija u cijelosti ostaje unutar zakupljene parcele 16,00 × 9,40 m
- - MJERODAVNO OPTEREĆENJE VJETROM: qp ≥ 1,20 kN/m² (udar 3 s ≈ 45 m/s) prema ovjerenoj projektnoj dokumentaciji lokacije i BAS EN 1991-1-4 sa BiH nacionalnim aneksom, uz primjenu faktora orografije za izloženi planinski vrh na 1076 m n.v. Koeficijent sile cf ≥ 1,5 pri 45° prema EN 1991-1-4 §7.3, osim ako se proračunom dokaže drugačije. Projektne sile po nosaču (GSN, γQ=1,5 / γG,fav=0,9): podizanje ≥27 kN, horizontalna sila ≥30 kN, moment prevrtanja ≥64 kNm. Mjerodavni su podizanje (uplift) i prevrtanje, a ne nosivost tla. NAPOMENA: kataloški nosač tipa A ima deklarisanu otpornost 31 m/s (0,52 kN/m²) pri 45° i 40 m/s (0,87 kN/m²) pri 15°/25°, što je ISPOD opterećenja ovog lokaliteta; Ponuđač je stoga dužan ponuditi konstrukciju dimenzionisanu i dokazanu za stvarno opterećenje lokaliteta, uz pisanu potvrdu proizvođača za konkretnu lokaciju (planinski vrh)
+ - gabariti PV polja po nosaču (2 reda × 2 modula, portret): širina polja 2305 mm (poprečna greda 2918 mm, bočni prepust 306,5 mm), dužina polja po nagibu 4576 mm (2 × 2278 mm, nepromijenjeno), horizontalna projekcija 3236 mm pri nagibu 45°; donja ivica panela na +1,50 m, gornja ivica na +4,74 m od nivoa terena — podignuto za 1,00 m u odnosu na raniju 2×6 izvedbu, jer manje opterećenje vjetra po nosaču to dopušta (v. proračun F.6)
+ - smještaj: nosači se temelje IZVAN ograđenog platoa, 400 mm južno od kote ograde (raspoloživi pojas 1950 mm); gornja (sjeverna) ivica panela je 2,84 m iznad kote ograde h=1,90 m. Ponuđač provjerava da konstrukcija u cijelosti ostaje unutar zakupljene parcele 16,00 × 9,40 m
+ - MJERODAVNO OPTEREĆENJE VJETROM: qp ≥ 1,20 kN/m² (udar 3 s ≈ 45 m/s) prema ovjerenoj projektnoj dokumentaciji lokacije i BAS EN 1991-1-4 sa BiH nacionalnim aneksom, uz primjenu faktora orografije za izloženi planinski vrh na 1076 m n.v. Koeficijent sile cf ≥ 1,5 pri 45° prema EN 1991-1-4 §7.3, osim ako se proračunom dokaže drugačije. Površina izloženosti vjetru 10,55 m² po nosaču (2305 × 4576 mm). Projektne sile po nosaču (GSN, γQ=1,5 / γG,fav=0,9): podizanje ≥18,1 kN, horizontalna sila ≥13,4 kN, moment prevrtanja ≥62,8 kNm. Mjerodavni su podizanje (uplift) i prevrtanje, a ne nosivost tla. NAPOMENA: kataloški nosač tipa A ima deklarisanu otpornost 31 m/s (0,52 kN/m²) pri 45° i 40 m/s (0,87 kN/m²) pri 15°/25°, što je ISPOD opterećenja ovog lokaliteta čak i za manje polje; Ponuđač je stoga dužan ponuditi konstrukciju dimenzionisanu i dokazanu za stvarno opterećenje lokaliteta, uz pisanu potvrdu proizvođača za konkretnu lokaciju (planinski vrh) ako se ipak nudi kataloški proizvod
  - materijal i izrada: konstrukcijski čelik S275JR (S355JR za stubove) prema EN 10025-2, šuplji profili prema EN 10219 — stubovi min. RHS 80×80×4, rigle min. RHS 60×40×3, ili bilo koji presjek za koji se proračunom dokaže najmanje jednak otporni moment; antikorozivna zaštita vrućim cinčanjem prema EN ISO 1461 min. 70 µm lokalno / 85 µm srednje (klasa korozivnosti C4); zavarivanje prema EN 1090-2 klasa izvedbe EXC2; CE označavanje i izjava o svojstvima prema EN 1090-1; konstrukcijski vijci M16 klase 8.8 prema EN 15048, pričvrsni pribor modula A2/A4 nehrđajući
  - spojni pribor: nehrđajući čelik A2/A4
- - uključeno ožičenje i povezivanje oba polja panela do PVDB distribucije</t>
+ - uključeno ožičenje i povezivanje sva tri polja panela do PVDB distribucije preko po-string DC odvodnika prenapona (v. Tačku 1.6a i crtež E-01): PV-1 i PV-2 paralelno na rutu 1, PV-3 samostalno na rutu 2</t>
         </is>
       </c>
       <c r="C12" s="79" t="inlineStr">
@@ -1328,7 +1328,7 @@
         </is>
       </c>
       <c r="D12" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="27" t="n"/>
       <c r="F12" s="27">
@@ -1475,9 +1475,9 @@
           <t>Isporuka i ugradnja sistema sidrenja nosive konstrukcije iz Tačke 1.1 u stijenu/beton, hemijskim (epoksidnim) ankerima.
  - tip: hemijski (epoksidni/vinilesterski) anker M16 ili M20 sa ETA odobrenjem za ugradnju u beton i/ili stijenu, vruće cinčan ili nehrđajući A4
  - broj: najmanje 2 ankera po temeljnoj traci, odnosno 4 ankera po nosaču (minimum 2 po traci zbog redundanse)
- - nosivost: karakteristična sila čupanja ≥30 kN po ankeru; dubina ugradnje prema ETA za konkretnu podlogu. Ukupna projektna sila podizanja po nosaču ≥27 kN (GSN)
+ - nosivost: karakteristična sila čupanja ≥30 kN po ankeru; dubina ugradnje prema ETA za konkretnu podlogu. Ukupna projektna sila podizanja po nosaču ≥18,1 kN (GSN); sila po traci od momenta prevrtanja ≥39,3 kN pri razmaku traka 1600 mm (v. proračun F.6)
  - dokazivanje: ispitivanje čupanjem (pull-out test) na najmanje 10 % ugrađenih ankera, minimalno 2 po nosaču, do 1,5 × projektne sile, uz zapisnik ovjeren od nadzornog organa
- - alternativa: livena U-anker sidra M16, dužine 320 mm, razmaka krakova 180 mm, sa pločama 50×50 mm i dvostrukim maticama, dozvoljena su SAMO uz gravitacioni temelj zapremine ≥1,14 m³ po nosaču (umjesto 0,81 m³)</t>
+ - alternativa: livena U-anker sidra M16, dužine 320 mm, razmaka krakova 180 mm, sa pločama 50×50 mm i dvostrukim maticama, dozvoljena su SAMO uz gravitacioni temelj zapremine ≥0,75 m³ po nosaču (tendovano 0,81 m³ po nosaču, v. Tačku 2.3) — momenat prevrtanja i dalje zahtijeva provjeru lokalnog istezanja trake, ne samo ukupne mase</t>
         </is>
       </c>
       <c r="C29" s="79" t="inlineStr">
@@ -1486,7 +1486,7 @@
         </is>
       </c>
       <c r="D29" s="79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E29" s="27" t="n"/>
       <c r="F29" s="27">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="D33" s="89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E33" s="41" t="n"/>
       <c r="F33" s="41">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="B34" s="91" t="inlineStr">
         <is>
-          <t>Isporuka i polaganje DC solarnog kabla 1×6 mm² (H1Z2Z2-K) od fotonaponskih panela do PVDB distribucije, uključujući MC4 konektore, obujmice i UV-otporne kanalice. NAPOMENA: završni priključak na ulaznu stezaljku iSSU modula izvesti presjekom 4 mm² prema izričitom zahtjevu proizvođača. Pad napona pri Imp 13,67 A i dužini 25 m iznosi 0,78 %. 2 nosača × 2 × 25,00 m</t>
+          <t>Isporuka i polaganje DC solarnog kabla 1×6 mm² (H1Z2Z2-K) od fotonaponskih panela do PVDB distribucije, uključujući MC4 konektore, obujmice i UV-otporne kanalice. NAPOMENA: završni priključak na ulaznu stezaljku iSSU modula izvesti presjekom 4 mm² prema izričitom zahtjevu proizvođača. Pad napona pri Imp 13,67 A i dužini 25 m iznosi 0,78 %. 3 nosača × 2 × 25,00 m</t>
         </is>
       </c>
       <c r="C34" s="89" t="inlineStr">
@@ -1582,7 +1582,7 @@
         </is>
       </c>
       <c r="D34" s="89" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="E34" s="41" t="n"/>
       <c r="F34" s="41">
@@ -1623,7 +1623,7 @@
       </c>
       <c r="B36" s="91" t="inlineStr">
         <is>
-          <t>Isporuka i ugradnja odvodnika prenapona DC, tip 2 (Iimp ≥5 kA, Ucpv ≥425 V), za svaki string, sa pripadajućim rastavnim osiguračima, u PVDB ormaru iz Tačke 1.6 ili u zasebnom kućištu min. IP55. Predvidjeti drugi komplet na strani polja panela zbog dužine DC trase od 25 m.</t>
+          <t>Isporuka i ugradnja odvodnika prenapona DC, tip 2 (Iimp ≥5 kA, Ucpv ≥425 V), za svaki string, sa pripadajućim rastavnim osiguračima, u PVDB ormaru iz Tačke 1.6 ili u zasebnom kućištu min. IP55. Po jedan komplet uz svako od tri polja panela (v. Tačku 1.1) zbog dužine DC trase od 25 m; PV-1 i PV-2 se spajaju paralelno prije PVDB rute 1, PV-3 ide samostalno na rutu 2 (v. crtež E-01).</t>
         </is>
       </c>
       <c r="C36" s="89" t="inlineStr">
@@ -1632,7 +1632,7 @@
         </is>
       </c>
       <c r="D36" s="89" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E36" s="41" t="n"/>
       <c r="F36" s="41">
@@ -1665,68 +1665,70 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="40" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="B38" s="90" t="inlineStr">
-        <is>
-          <t>OPCIJA (alternativna ponuda — cijena se iskazuje posebno i NE ulazi u zbir Tačke 1): Isporuka i montaža TRI nosača sa po 4 fotonaponska modula (3 × 4 = 12 modula, ista ukupna snaga 7,02 kWp) umjesto dva nosača sa po 6 modula. Površina izloženosti vjetru po nosaču smanjuje se sa 15,91 m² na 7,95 m² (−50 %), čime se približno prepolovljuju sila podizanja i moment prevrtanja po temelju, uz zadržavanje nagiba 45°. Uključuje treći komplet temelja, sidrenja i uzemljenja. Kupac zadržava pravo izbora između osnovne i alternativne izvedbe.</t>
-        </is>
-      </c>
-      <c r="C38" s="89" t="inlineStr">
-        <is>
-          <t>kpl</t>
-        </is>
-      </c>
-      <c r="D38" s="89" t="n">
-        <v>1</v>
-      </c>
-      <c r="E38" s="41" t="n"/>
-      <c r="F38" s="41" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="92" t="inlineStr">
+      <c r="A38" s="92" t="inlineStr">
         <is>
           <t>UKUPNO 1 — NOSAČI ZA FOTONAPONSKE PANELE:</t>
         </is>
       </c>
-      <c r="B39" s="93" t="n"/>
-      <c r="C39" s="93" t="n"/>
-      <c r="D39" s="93" t="n"/>
-      <c r="E39" s="94" t="n"/>
-      <c r="F39" s="67">
-        <f>SUM(F12:F38)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" ht="24" customHeight="1" s="69"/>
+      <c r="B38" s="93" t="n"/>
+      <c r="C38" s="93" t="n"/>
+      <c r="D38" s="93" t="n"/>
+      <c r="E38" s="94" t="n"/>
+      <c r="F38" s="67">
+        <f>SUM(F12:F37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40" ht="24" customHeight="1" s="69">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>GRAĐEVINSKI RADOVI</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
+      <c r="F40" s="5" t="n"/>
+    </row>
     <row r="41" ht="24" customHeight="1" s="69">
-      <c r="A41" s="3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>GRAĐEVINSKI RADOVI</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="n"/>
-      <c r="D41" s="5" t="n"/>
-      <c r="E41" s="5" t="n"/>
-      <c r="F41" s="5" t="n"/>
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="B41" s="77" t="inlineStr">
+        <is>
+          <t>Iskop zemlje IV-V kategorije za temeljne trake nosača. Iskop cca 1,59 m3 za svaku temeljnu traku. 3 nosača × 2 trake × 1,59 m3</t>
+        </is>
+      </c>
+      <c r="C41" s="76" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D41" s="76" t="n">
+        <v>9.539999999999999</v>
+      </c>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8">
+        <f>IF(AND(D41&lt;&gt;"",E41&lt;&gt;""),D41*E41,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>2.1</t>
-        </is>
-      </c>
-      <c r="B42" s="77" t="inlineStr">
-        <is>
-          <t>Iskop zemlje IV-V kategorije za temeljne trake nosača. Iskop cca 1,59 m3 za svaku temeljnu traku. 2 nosača × 2 trake × 1,59 m3</t>
+          <t>2.2</t>
+        </is>
+      </c>
+      <c r="B42" s="78" t="inlineStr">
+        <is>
+          <t>Zatrpavanje rova zemljom od iskopa uz nabijanje u slojevima. 3 nosača × 2 trake × 1,10 m3</t>
         </is>
       </c>
       <c r="C42" s="76" t="inlineStr">
@@ -1735,7 +1737,7 @@
         </is>
       </c>
       <c r="D42" s="76" t="n">
-        <v>6.36</v>
+        <v>6.6</v>
       </c>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8">
@@ -1746,12 +1748,12 @@
     <row r="43" ht="24" customHeight="1" s="69">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>2.2</t>
-        </is>
-      </c>
-      <c r="B43" s="78" t="inlineStr">
-        <is>
-          <t>Zatrpavanje rova zemljom od iskopa uz nabijanje u slojevima. 2 nosača × 2 trake × 1,10 m3</t>
+          <t>2.2a</t>
+        </is>
+      </c>
+      <c r="B43" s="77" t="inlineStr">
+        <is>
+          <t>Odvoz i zbrinjavanje viška materijala od iskopa do deponije udaljene do 20 km.</t>
         </is>
       </c>
       <c r="C43" s="76" t="inlineStr">
@@ -1760,7 +1762,7 @@
         </is>
       </c>
       <c r="D43" s="76" t="n">
-        <v>4.4</v>
+        <v>2.94</v>
       </c>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8">
@@ -1771,12 +1773,12 @@
     <row r="44" ht="156" customHeight="1" s="69">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>2.2a</t>
+          <t>2.2b</t>
         </is>
       </c>
       <c r="B44" s="77" t="inlineStr">
         <is>
-          <t>Odvoz i zbrinjavanje viška materijala od iskopa do deponije udaljene do 20 km.</t>
+          <t>Nabavka materijala, transport i ugradnja betona C10 ispod temeljnih traka, prema zahtjevima proizvođača. 3 nosača × 2 trake × 0,094 m3</t>
         </is>
       </c>
       <c r="C44" s="76" t="inlineStr">
@@ -1785,7 +1787,7 @@
         </is>
       </c>
       <c r="D44" s="76" t="n">
-        <v>1.96</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8">
@@ -1796,12 +1798,13 @@
     <row r="45" ht="24" customHeight="1" s="69">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>2.2b</t>
+          <t>2.3</t>
         </is>
       </c>
       <c r="B45" s="77" t="inlineStr">
         <is>
-          <t>Nabavka materijala, transport i ugradnja betona C10 ispod temeljnih traka, prema zahtjevima proizvođača. 2 nosača × 2 trake × 0,094 m3</t>
+          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C25, uz upotrebu oplate za nadzemni dio. Traka je širine 450 mm (550 mm u dnu), dužine 3300 mm i dubine 900 mm, postavljena u pravcu SJEVER-JUG (u pravcu nagiba panela), na osovinskom razmaku 1600 mm, sve prema nacrtu proizvođača nosača. Armiranje rebrastom armaturom Ø10, granica razvlačenja 335 MPa, prema specifikaciji proizvođača (poz. R01–R04, cca 19,53 kg po traci, ukupno cca 78 kg), zaštitni sloj betona 50 mm — što ulazi u cijenu betona. Prije betoniranja pravilno pozicionirati anker vijke iz Tačke 1.2 (vezani za armaturu poz. R04), uzemljivačku traku i PEHD cijevi. Ugradnja betona pervibratorom, njega betona vlaženjem najmanje 3 dana, dozvoljeno odstupanje ±3 mm. NAPOMENA: nosivost tla ispod temelja (fak) mora iznositi najmanje 100 kPa, a osnovna brzina vjetra za nagib 45° iznosi 31 m/s (3 s udar). Proizvođač izričito zahtijeva da se za lokacije na planinskim vrhovima projekat temelja ponovo provjeri i prilagodi. 3 nosača × 2 trake × 0,407 m3.  Obračun po ostvarenom m3 betona.
+IZMJENA — BETON I ARMATURA: beton klase C30/37, klase izloženosti XC4 + XF3 prema BAS EN 206, sa aerantom 4–6 %, Dmax 16, konzistencija S3; podložni beton C12/15 d=50 mm; armatura B500B, zaštitni sloj ≥50 mm. Klasa XF3 je mjerodavna zbog cikličnog smrzavanja i odmrzavanja u vlažnom stanju na 1076 m n.v. Temeljna spojnica mora biti ispod dubine smrzavanja za lokalitet, koju Ponuđač navodi u ponudi. Dubina trake prema ovjerenom statičkom proračunu iz Tačke 1.3.</t>
         </is>
       </c>
       <c r="C45" s="76" t="inlineStr">
@@ -1810,7 +1813,7 @@
         </is>
       </c>
       <c r="D45" s="76" t="n">
-        <v>0.38</v>
+        <v>2.44</v>
       </c>
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="8">
@@ -1821,24 +1824,22 @@
     <row r="46" s="69">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="B46" s="77" t="inlineStr">
-        <is>
-          <t>Nabavka materijala, transport i betoniranje DVIJE temeljne trake po nosaču, betonom C25, uz upotrebu oplate za nadzemni dio. Traka je širine 450 mm (550 mm u dnu), dužine 3300 mm i dubine 900 mm, postavljena u pravcu SJEVER-JUG (u pravcu nagiba panela), na osovinskom razmaku 2600 mm, sve prema nacrtu proizvođača nosača. Armiranje rebrastom armaturom Ø10, granica razvlačenja 335 MPa, prema specifikaciji proizvođača (poz. R01–R04, cca 19,53 kg po traci, ukupno cca 78 kg), zaštitni sloj betona 50 mm — što ulazi u cijenu betona. Prije betoniranja pravilno pozicionirati anker vijke iz Tačke 1.2 (vezani za armaturu poz. R04), uzemljivačku traku i PEHD cijevi. Ugradnja betona pervibratorom, njega betona vlaženjem najmanje 3 dana, dozvoljeno odstupanje ±3 mm. NAPOMENA: nosivost tla ispod temelja (fak) mora iznositi najmanje 100 kPa, a osnovna brzina vjetra za nagib 45° iznosi 31 m/s (3 s udar). Proizvođač izričito zahtijeva da se za lokacije na planinskim vrhovima projekat temelja ponovo provjeri i prilagodi. 2 nosača × 2 trake × 0,407 m3.  Obračun po ostvarenom m3 betona.
-IZMJENA — BETON I ARMATURA: beton klase C30/37, klase izloženosti XC4 + XF3 prema BAS EN 206, sa aerantom 4–6 %, Dmax 16, konzistencija S3; podložni beton C12/15 d=50 mm; armatura B500B, zaštitni sloj ≥50 mm. Klasa XF3 je mjerodavna zbog cikličnog smrzavanja i odmrzavanja u vlažnom stanju na 1076 m n.v. Temeljna spojnica mora biti ispod dubine smrzavanja za lokalitet, koju Ponuđač navodi u ponudi. Dubina trake prema ovjerenom statičkom proračunu iz Tačke 1.3.</t>
-        </is>
-      </c>
-      <c r="C46" s="76" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
-      <c r="D46" s="76" t="n">
-        <v>1.63</v>
-      </c>
-      <c r="E46" s="8" t="n"/>
+          <t>2.4</t>
+        </is>
+      </c>
+      <c r="B46" s="97" t="inlineStr">
+        <is>
+          <t>Obrada vidljivih strana i gornje površine temeljnih traka cementnim malterom u nagibu 1,0 %, zaglađeno do crnog sjaja.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>12</v>
+      </c>
       <c r="F46" s="8">
         <f>IF(AND(D46&lt;&gt;"",E46&lt;&gt;""),D46*E46,"")</f>
         <v/>
@@ -1847,125 +1848,118 @@
     <row r="47" s="69">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>2.4</t>
-        </is>
-      </c>
-      <c r="B47" s="97" t="inlineStr">
-        <is>
-          <t>Obrada vidljivih strana i gornje površine temeljnih traka cementnim malterom u nagibu 1,0 %, zaglađeno do crnog sjaja.</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="D47" t="n">
-        <v>12</v>
-      </c>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="B47" s="78" t="inlineStr">
+        <is>
+          <t>Ostali sitni građevinski i potrošni materijal.</t>
+        </is>
+      </c>
+      <c r="C47" s="76" t="inlineStr">
+        <is>
+          <t>paušal</t>
+        </is>
+      </c>
+      <c r="D47" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="8" t="n"/>
       <c r="F47" s="8">
         <f>IF(AND(D47&lt;&gt;"",E47&lt;&gt;""),D47*E47,"")</f>
         <v/>
       </c>
     </row>
     <row r="48" s="69">
-      <c r="A48" s="6" t="inlineStr">
-        <is>
-          <t>2.5</t>
-        </is>
-      </c>
-      <c r="B48" s="78" t="inlineStr">
-        <is>
-          <t>Ostali sitni građevinski i potrošni materijal.</t>
-        </is>
-      </c>
-      <c r="C48" s="76" t="inlineStr">
-        <is>
-          <t>paušal</t>
-        </is>
-      </c>
-      <c r="D48" s="76" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" s="8" t="n"/>
-      <c r="F48" s="8">
-        <f>IF(AND(D48&lt;&gt;"",E48&lt;&gt;""),D48*E48,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" s="69">
-      <c r="A49" s="15" t="inlineStr">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>UKUPNO 2 — GRAĐEVINSKI RADOVI ZA NOSAČE FN PANELA:</t>
         </is>
       </c>
-      <c r="B49" s="16" t="n"/>
-      <c r="C49" s="16" t="n"/>
-      <c r="D49" s="16" t="n"/>
-      <c r="E49" s="17" t="n"/>
-      <c r="F49" s="10">
-        <f>SUM(F42:F48)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="95" t="inlineStr">
+      <c r="B48" s="16" t="n"/>
+      <c r="C48" s="16" t="n"/>
+      <c r="D48" s="16" t="n"/>
+      <c r="E48" s="17" t="n"/>
+      <c r="F48" s="10">
+        <f>SUM(F41:F47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49" s="69"/>
+    <row r="50">
+      <c r="A50" s="95" t="inlineStr">
         <is>
           <t>UKUPNO LOT 1 — NOSAČI ZA FOTONAPONSKE PANELE (bez PDV-a):</t>
         </is>
       </c>
-      <c r="B51" s="16" t="n"/>
-      <c r="C51" s="16" t="n"/>
-      <c r="D51" s="17" t="n"/>
-      <c r="E51" s="17" t="n"/>
-      <c r="F51" s="11">
-        <f>F39+F49</f>
-        <v/>
-      </c>
+      <c r="B50" s="16" t="n"/>
+      <c r="C50" s="16" t="n"/>
+      <c r="D50" s="17" t="n"/>
+      <c r="E50" s="17" t="n"/>
+      <c r="F50" s="11">
+        <f>F38+F48</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51"/>
+    <row r="52">
+      <c r="A52" s="98" t="inlineStr">
+        <is>
+          <t>REKAPITULACIJA — LOT 1</t>
+        </is>
+      </c>
+      <c r="B52" s="103" t="n"/>
+      <c r="C52" s="103" t="n"/>
+      <c r="D52" s="103" t="n"/>
+      <c r="E52" s="104" t="n"/>
+      <c r="F52" s="100" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="98" t="inlineStr">
-        <is>
-          <t>REKAPITULACIJA — LOT 1</t>
+      <c r="A53" s="101" t="inlineStr">
+        <is>
+          <t>UKUPNO LOT 1 (bez PDV-a):</t>
         </is>
       </c>
       <c r="B53" s="103" t="n"/>
       <c r="C53" s="103" t="n"/>
       <c r="D53" s="103" t="n"/>
       <c r="E53" s="104" t="n"/>
-      <c r="F53" s="100" t="n"/>
+      <c r="F53" s="102">
+        <f>F50</f>
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="101" t="inlineStr">
         <is>
-          <t>UKUPNO LOT 1 (bez PDV-a):</t>
+          <t>Popust (%):</t>
         </is>
       </c>
       <c r="B54" s="103" t="n"/>
       <c r="C54" s="103" t="n"/>
       <c r="D54" s="103" t="n"/>
       <c r="E54" s="104" t="n"/>
-      <c r="F54" s="102">
-        <f>F51</f>
-        <v/>
-      </c>
+      <c r="F54" s="102" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="101" t="inlineStr">
         <is>
-          <t>Popust (%):</t>
+          <t>UKUPNO LOT 1 sa popustom (bez PDV-a):</t>
         </is>
       </c>
       <c r="B55" s="103" t="n"/>
       <c r="C55" s="103" t="n"/>
       <c r="D55" s="103" t="n"/>
       <c r="E55" s="104" t="n"/>
-      <c r="F55" s="102" t="n"/>
+      <c r="F55" s="102">
+        <f>F53*(1-IF(F54="",0,F54/100))</f>
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="101" t="inlineStr">
         <is>
-          <t>UKUPNO LOT 1 sa popustom (bez PDV-a):</t>
+          <t>PDV 17%:</t>
         </is>
       </c>
       <c r="B56" s="103" t="n"/>
@@ -1973,40 +1967,26 @@
       <c r="D56" s="103" t="n"/>
       <c r="E56" s="104" t="n"/>
       <c r="F56" s="102">
-        <f>F54*(1-IF(F55="",0,F55/100))</f>
+        <f>F55*0.17</f>
         <v/>
       </c>
     </row>
     <row r="57" ht="24" customHeight="1" s="69">
-      <c r="A57" s="101" t="inlineStr">
-        <is>
-          <t>PDV 17%:</t>
+      <c r="A57" s="98" t="inlineStr">
+        <is>
+          <t>UKUPNO LOT 1 sa PDV-om:</t>
         </is>
       </c>
       <c r="B57" s="103" t="n"/>
       <c r="C57" s="103" t="n"/>
       <c r="D57" s="103" t="n"/>
       <c r="E57" s="104" t="n"/>
-      <c r="F57" s="102">
-        <f>F56*0.17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="98" t="inlineStr">
-        <is>
-          <t>UKUPNO LOT 1 sa PDV-om:</t>
-        </is>
-      </c>
-      <c r="B58" s="103" t="n"/>
-      <c r="C58" s="103" t="n"/>
-      <c r="D58" s="103" t="n"/>
-      <c r="E58" s="104" t="n"/>
-      <c r="F58" s="100">
-        <f>F56+F57</f>
-        <v/>
-      </c>
-    </row>
+      <c r="F57" s="100">
+        <f>F55+F56</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58"/>
     <row r="59" ht="24" customHeight="1" s="69"/>
     <row r="83" ht="24" customHeight="1" s="69"/>
     <row r="84" ht="24" customHeight="1" s="69"/>
@@ -4104,7 +4084,7 @@
       <c r="D132" s="9" t="n"/>
       <c r="E132" s="9" t="n"/>
       <c r="F132" s="8">
-        <f>'LOT 1'!F51</f>
+        <f>'LOT 1'!F50</f>
         <v/>
       </c>
     </row>

</xml_diff>